<commit_message>
feat(productos): Kit de Tareas Bar v2.0 (342 tareas, 07 con secciones propias) y Dark Kitchen v2.0 (331, 08 en vocabulario delivery) — motor 2.4 + contenido propio; idempotencia 0, cache 133/133, censo 0, gate offline 11/11
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-bar/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-bar/01-apertura-cierre.xlsx
@@ -12,8 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cierre Barra" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$B$44</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Apertura Barra'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Apertura Barra'!$A$1:$G$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Cierre Barra'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Cierre Barra'!$A$1:$G$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,8 +97,22 @@
       <color rgb="00999999"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFD700"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -136,6 +153,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8E1"/>
         <bgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
   </fills>
@@ -209,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -266,6 +293,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,92 +737,223 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="33" t="inlineStr">
         <is>
           <t>01 — Apertura y Cierre · Bar / Cocktails</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Cómo usar esta plantilla:</t>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>Cómo usar esta plantilla</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>▸ Imprime el checklist del turno correspondiente cada día</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+    <row r="7" ht="16" customHeight="1">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>▸ El responsable de turno marca cada tarea al completarla</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="3" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>▸ Al finalizar el turno, firma y entrega al siguiente responsable</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Personalización:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>Personalización</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>▸ Las celdas verdes son editables — ajusta responsables y horarios</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>▸ Añade tareas específicas de tu bar en las filas vacías</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>▸ Borra las tareas que no apliquen a tu negocio</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>Cómo cuenta el contador</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-bar · info@aichef.pro</t>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>▸ Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>▸ «N/A» = no aplica en tu local: esa tarea SALE del total (no la borres, márcala N/A). «—» = no hecha: sigue contando como pendiente y baja el porcentaje, que es de lo que se trata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>▸ El denominador cuenta las tareas escritas en la columna «Tarea», no un número fijo: si añades o borras tareas, el total se ajusta solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>Filas libres</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>▸ Al final de cada tabla hay 5 filas verdes libres DENTRO del rango que cuenta el contador: escribe ahí tus tareas propias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>▸ Si necesitas más, inserta filas DENTRO de la tabla (clic derecho → Insertar), nunca por debajo de la última: lo que se escriba fuera del rango no lo cuenta nadie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>Protección de la hoja</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t>▸ Las hojas con fórmulas van protegidas SIN contraseña: las celdas de entrada (las verdes) están desbloqueadas y los cálculos no se pisan por accidente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>▸ Puedes insertar y borrar filas con la protección puesta. Para cambiar la estructura: Revisar → Desproteger hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>Se conecta con</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>▸ 08-apertura-cierre-negocio.xlsx — checklist del LOCAL completo: es el MARCO del día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="B34" s="35" t="inlineStr">
+        <is>
+          <t>▸ 01-apertura-cierre.xlsx — el mismo día con el DETALLE por área (barra).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>▸ 09-apertura-cierre-caja.xlsx — la CAJA: fondo, recuento por denominaciones, Z del TPV y descuadre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>▸ Orden de uso: local → áreas → caja. Cada fichero cubre un nivel: el de negocio marca el HITO (encender, abrir, cerrar), el de áreas detalla CÓMO se hace en cada zona y el de caja lleva el DINERO. Si una tarea aparece en dos, es a propósito: una es el hito y la otra el detalle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>▸ Estás en 01-apertura-cierre.xlsx: es una capa MÁS, no una repetición — el marco del día está en 08-apertura-cierre-negocio.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Bar / Cocktails · AI Chef Pro · aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="34" t="inlineStr">
+        <is>
+          <t>Contacto: info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="34" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-bar · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -753,7 +978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -818,802 +1043,1029 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HIGIENE PERSONAL</t>
+        </is>
+      </c>
+      <c r="B5" s="37" t="n"/>
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="37" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="F5" s="37" t="n"/>
+      <c r="G5" s="38" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Uniforme y delantal limpios, pelo recogido y calzado antideslizante (detrás de la barra el suelo se moja siempre)</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F6" s="43" t="n"/>
+      <c r="G6" s="44" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Sin anillos, reloj ni pulseras; uñas cortas, limpias y sin esmalte: se manipulan hielo, cítricos y garnish sin guante</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="n"/>
+      <c r="G7" s="44" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Heridas y cortes cubiertos con apósito impermeable de color visible y guante encima</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="n"/>
+      <c r="G8" s="44" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Lavado de manos al entrar y en cada cambio de tarea; lavamanos de barra con jabón, papel y agua caliente</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="n"/>
+      <c r="G9" s="44" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Declarar síntomas digestivos o respiratorios: quien los tenga no manipula hielo ni alimentos</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>Head Bartender</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="n"/>
+      <c r="G10" s="44" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="45" t="n"/>
+      <c r="B11" s="45" t="n"/>
+      <c r="C11" s="45" t="n"/>
+      <c r="D11" s="45" t="n"/>
+      <c r="E11" s="45" t="n"/>
+      <c r="F11" s="45" t="n"/>
+      <c r="G11" s="45" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  Mise en Place de Barra</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n"/>
-      <c r="C5" s="30" t="n"/>
-      <c r="D5" s="30" t="n"/>
-      <c r="E5" s="30" t="n"/>
-      <c r="F5" s="30" t="n"/>
-      <c r="G5" s="31" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B12" s="37" t="n"/>
+      <c r="C12" s="37" t="n"/>
+      <c r="D12" s="37" t="n"/>
+      <c r="E12" s="37" t="n"/>
+      <c r="F12" s="37" t="n"/>
+      <c r="G12" s="38" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>Encender iluminación de barra y ambiente</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E13" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="15" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="F13" s="43" t="n"/>
+      <c r="G13" s="44" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>Encender sistema de música / ambientación sonora</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="15" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="F14" s="43" t="n"/>
+      <c r="G14" s="44" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>Verificar limpieza de barra, mostrador y taburetes</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E15" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="15" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Encender cámaras de barra (verificar temperatura 2-4 °C)</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="F15" s="43" t="n"/>
+      <c r="G15" s="44" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Comprobar que las cámaras y el botellero de barra han funcionado toda la noche y registrar temperatura (2-4 °C) — anota la lectura: ____ °C. Si hay desviación, no sirvas el producto hasta valorarlo</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="15" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="F16" s="43" t="n"/>
+      <c r="G16" s="44" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>Preparar mise en place de cítricos (rodajas limón, lima, naranja)</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E17" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="15" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="F17" s="43" t="n"/>
+      <c r="G17" s="44" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>Preparar garnish: aceitunas, cerezas, piel de cítricos, hierbas frescas</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="15" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="32" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="F18" s="43" t="n"/>
+      <c r="G18" s="44" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>Llenar cubetas de hielo (cubos, hielo pilé, bloques grandes)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E19" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="15" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="F19" s="43" t="n"/>
+      <c r="G19" s="44" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>Verificar stock de hielo (mínimo para el turno: 30-50 kg)</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E20" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="15" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="F20" s="43" t="n"/>
+      <c r="G20" s="44" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>Preparar speed rail con botellas más usadas</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E21" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="15" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="32" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="F21" s="43" t="n"/>
+      <c r="G21" s="44" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t>Verificar stock de zumos naturales (preparar si falta)</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E22" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="F22" s="43" t="n"/>
+      <c r="G22" s="44" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="40" t="inlineStr">
         <is>
           <t>Preparar jarabes del día (simple, gomme, especiales)</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E23" s="42" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="15" t="n"/>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="F23" s="43" t="n"/>
+      <c r="G23" s="44" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="45" t="n"/>
+      <c r="C24" s="45" t="n"/>
+      <c r="D24" s="45" t="n"/>
+      <c r="E24" s="45" t="n"/>
+      <c r="F24" s="45" t="n"/>
+      <c r="G24" s="45" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cristalería y Material</t>
         </is>
       </c>
-      <c r="B18" s="30" t="n"/>
-      <c r="C18" s="30" t="n"/>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="30" t="n"/>
-      <c r="G18" s="31" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="37" t="n"/>
+      <c r="D25" s="37" t="n"/>
+      <c r="E25" s="37" t="n"/>
+      <c r="F25" s="37" t="n"/>
+      <c r="G25" s="38" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>Pulir cristalería: copas de vino, copas cóctel, vasos old fashioned</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C26" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E26" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="15" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="F26" s="43" t="n"/>
+      <c r="G26" s="44" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>Verificar stock de cristalería limpia (mínimo 2x capacidad)</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D27" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E27" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="15" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="32" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="F27" s="43" t="n"/>
+      <c r="G27" s="44" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>Preparar coctelera, jigger, colador, bar spoon, muddler</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C28" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D28" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E28" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="15" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="32" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="F28" s="43" t="n"/>
+      <c r="G28" s="44" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="39" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>Verificar stock de pajitas, servilletas y posavasos</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C29" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D29" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E29" s="42" t="inlineStr">
         <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="15" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="32" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="F29" s="43" t="n"/>
+      <c r="G29" s="44" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>Preparar tickets de comandas / tablet de pedidos</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C30" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D30" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E30" s="42" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="15" t="n"/>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="F30" s="43" t="n"/>
+      <c r="G30" s="44" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="45" t="n"/>
+      <c r="B31" s="45" t="n"/>
+      <c r="C31" s="45" t="n"/>
+      <c r="D31" s="45" t="n"/>
+      <c r="E31" s="45" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="45" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">  Máquina de Café</t>
         </is>
       </c>
-      <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
-      <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
-      <c r="F25" s="30" t="n"/>
-      <c r="G25" s="31" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="32" t="n">
-        <v>17</v>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="37" t="n"/>
+      <c r="G32" s="38" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="39" t="n">
+        <v>22</v>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
         <is>
           <t>Encender máquina de espresso (precalentar 20 min)</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C33" s="41" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D33" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E33" s="42" t="inlineStr">
         <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="15" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="32" t="n">
-        <v>18</v>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="F33" s="43" t="n"/>
+      <c r="G33" s="44" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="39" t="n">
+        <v>23</v>
+      </c>
+      <c r="B34" s="40" t="inlineStr">
         <is>
           <t>Purgar grupo (agua caliente 10 segundos por grupo)</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C34" s="41" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D34" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E34" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="15" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="32" t="n">
-        <v>19</v>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Verificar molienda y calibrar (espresso 25-30 seg, 25-30 ml)</t>
-        </is>
-      </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="F34" s="43" t="n"/>
+      <c r="G34" s="44" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="39" t="n">
+        <v>24</v>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>Verificar molienda y calibrar (espresso 25-30 segundos, 25-30 ml)</t>
+        </is>
+      </c>
+      <c r="C35" s="41" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D35" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E35" s="42" t="inlineStr">
         <is>
           <t>16:05</t>
         </is>
       </c>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="15" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="32" t="n">
-        <v>20</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="F35" s="43" t="n"/>
+      <c r="G35" s="44" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="n">
+        <v>25</v>
+      </c>
+      <c r="B36" s="40" t="inlineStr">
         <is>
           <t>Verificar stock de leche (entera, avena, soja)</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C36" s="41" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D36" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E36" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="15" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="32" t="n">
-        <v>21</v>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="F36" s="43" t="n"/>
+      <c r="G36" s="44" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="B37" s="40" t="inlineStr">
         <is>
           <t>Limpiar boquilla de vapor</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C37" s="41" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D37" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E37" s="42" t="inlineStr">
         <is>
           <t>16:05</t>
         </is>
       </c>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="15" t="n"/>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="F37" s="43" t="n"/>
+      <c r="G37" s="44" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="n"/>
+      <c r="B38" s="45" t="n"/>
+      <c r="C38" s="45" t="n"/>
+      <c r="D38" s="45" t="n"/>
+      <c r="E38" s="45" t="n"/>
+      <c r="F38" s="45" t="n"/>
+      <c r="G38" s="45" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apertura Terraza (si aplica)</t>
         </is>
       </c>
-      <c r="B32" s="30" t="n"/>
-      <c r="C32" s="30" t="n"/>
-      <c r="D32" s="30" t="n"/>
-      <c r="E32" s="30" t="n"/>
-      <c r="F32" s="30" t="n"/>
-      <c r="G32" s="31" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="32" t="n">
-        <v>22</v>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B39" s="37" t="n"/>
+      <c r="C39" s="37" t="n"/>
+      <c r="D39" s="37" t="n"/>
+      <c r="E39" s="37" t="n"/>
+      <c r="F39" s="37" t="n"/>
+      <c r="G39" s="38" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="39" t="n">
+        <v>27</v>
+      </c>
+      <c r="B40" s="40" t="inlineStr">
         <is>
           <t>Sacar mobiliario de terraza (mesas, sillas, sombrillas)</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C40" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D40" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E40" s="42" t="inlineStr">
         <is>
           <t>15:30</t>
         </is>
       </c>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="15" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="32" t="n">
-        <v>23</v>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="F40" s="43" t="n"/>
+      <c r="G40" s="44" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="39" t="n">
+        <v>28</v>
+      </c>
+      <c r="B41" s="40" t="inlineStr">
         <is>
           <t>Limpiar mesas y sillas de terraza</t>
         </is>
       </c>
-      <c r="C34" s="20" t="inlineStr">
+      <c r="C41" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D41" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E41" s="42" t="inlineStr">
         <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="32" t="n">
-        <v>24</v>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="F41" s="43" t="n"/>
+      <c r="G41" s="44" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="39" t="n">
+        <v>29</v>
+      </c>
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>Colocar ceniceros, cartas y servilleteros</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C42" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D42" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E42" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F35" s="14" t="n"/>
-      <c r="G35" s="15" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="32" t="n">
-        <v>25</v>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="F42" s="43" t="n"/>
+      <c r="G42" s="44" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="39" t="n">
+        <v>30</v>
+      </c>
+      <c r="B43" s="40" t="inlineStr">
         <is>
           <t>Verificar iluminación exterior</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
+      <c r="C43" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D43" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E43" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="15" t="n"/>
-    </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="F43" s="43" t="n"/>
+      <c r="G43" s="44" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="48" t="n"/>
+      <c r="B44" s="49" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="42" t="n"/>
+      <c r="E44" s="42" t="n"/>
+      <c r="F44" s="43" t="n"/>
+      <c r="G44" s="44" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="48" t="n"/>
+      <c r="B45" s="49" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="42" t="n"/>
+      <c r="E45" s="42" t="n"/>
+      <c r="F45" s="43" t="n"/>
+      <c r="G45" s="44" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="48" t="n"/>
+      <c r="B46" s="49" t="n"/>
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="42" t="n"/>
+      <c r="E46" s="42" t="n"/>
+      <c r="F46" s="43" t="n"/>
+      <c r="G46" s="44" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="48" t="n"/>
+      <c r="B47" s="49" t="n"/>
+      <c r="C47" s="41" t="n"/>
+      <c r="D47" s="42" t="n"/>
+      <c r="E47" s="42" t="n"/>
+      <c r="F47" s="43" t="n"/>
+      <c r="G47" s="44" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="48" t="n"/>
+      <c r="B48" s="49" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="42" t="n"/>
+      <c r="E48" s="42" t="n"/>
+      <c r="F48" s="43" t="n"/>
+      <c r="G48" s="44" t="n"/>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="D39" s="21">
-        <f>COUNTIF(F5:F37,"✓")</f>
+      <c r="D50" s="21">
+        <f>COUNTIFS(B5:B48,"?*",F5:F48,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F39" s="21">
-        <f>COUNTIF(B5:B37,"?*")</f>
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="F50" s="21">
+        <f>COUNTIF(B5:B48,"?*")-COUNTIF(F5:F48,"N/A")</f>
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>Verificado por:</t>
         </is>
       </c>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="30" t="n"/>
-      <c r="D41" s="31" t="n"/>
-      <c r="E41" s="21" t="inlineStr">
+      <c r="B52" s="50" t="n"/>
+      <c r="C52" s="30" t="n"/>
+      <c r="D52" s="31" t="n"/>
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="F41" s="15" t="n"/>
-      <c r="G41" s="31" t="n"/>
-    </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="23" t="inlineStr">
+      <c r="F52" s="50" t="n"/>
+      <c r="G52" s="31" t="n"/>
+    </row>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>— Kit de Tareas Recurrentes · Bar / Cocktails · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="10">
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F52:G52"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B52:D52"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G37">
+  <conditionalFormatting sqref="A5:G48">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F19 F20 F21 F22 F23 F26 F27 F28 F29 F30 F33 F34 F35 F36 F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F26 F27 F28 F29 F30 F33 F34 F35 F36 F37 F40 F41 F42 F43 F44 F45 F46 F47 F48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1637,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1702,748 +2154,844 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cierre de Servicio</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n"/>
-      <c r="C5" s="30" t="n"/>
-      <c r="D5" s="30" t="n"/>
-      <c r="E5" s="30" t="n"/>
-      <c r="F5" s="30" t="n"/>
-      <c r="G5" s="31" t="n"/>
+      <c r="B5" s="37" t="n"/>
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="37" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="F5" s="37" t="n"/>
+      <c r="G5" s="38" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="n">
+      <c r="A6" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>Última ronda: avisar a clientes 30 min antes de cierre</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="42" t="inlineStr">
         <is>
           <t>01:30</t>
         </is>
       </c>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="F6" s="43" t="n"/>
+      <c r="G6" s="44" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="32" t="n">
+      <c r="A7" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>Recoger cristalería de mesas y barra</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="43" t="n"/>
+      <c r="G7" s="44" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="n">
+      <c r="A8" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>Vaciar y limpiar cubetas de hielo</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="F8" s="43" t="n"/>
+      <c r="G8" s="44" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="n">
+      <c r="A9" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="40" t="inlineStr">
         <is>
           <t>Guardar mise en place de cítricos y garnish (film, cámara)</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="F9" s="43" t="n"/>
+      <c r="G9" s="44" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="n">
+      <c r="A10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>Guardar jarabes y zumos en cámara (tapar, etiquetar)</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="F10" s="43" t="n"/>
+      <c r="G10" s="44" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="n">
+      <c r="A11" s="39" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>Tapar botellas abiertas de speed rail</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="15" t="n"/>
+      <c r="F11" s="43" t="n"/>
+      <c r="G11" s="44" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="n">
+      <c r="A12" s="39" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>Limpiar coctelera, jigger, colador y utensilios</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="15" t="n"/>
-    </row>
-    <row r="13"/>
+      <c r="F12" s="43" t="n"/>
+      <c r="G12" s="44" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="45" t="n"/>
+      <c r="B13" s="45" t="n"/>
+      <c r="C13" s="45" t="n"/>
+      <c r="D13" s="45" t="n"/>
+      <c r="E13" s="45" t="n"/>
+      <c r="F13" s="45" t="n"/>
+      <c r="G13" s="45" t="n"/>
+    </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  Limpieza de Barra</t>
         </is>
       </c>
-      <c r="B14" s="30" t="n"/>
-      <c r="C14" s="30" t="n"/>
-      <c r="D14" s="30" t="n"/>
-      <c r="E14" s="30" t="n"/>
-      <c r="F14" s="30" t="n"/>
-      <c r="G14" s="31" t="n"/>
+      <c r="B14" s="37" t="n"/>
+      <c r="C14" s="37" t="n"/>
+      <c r="D14" s="37" t="n"/>
+      <c r="E14" s="37" t="n"/>
+      <c r="F14" s="37" t="n"/>
+      <c r="G14" s="38" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="n">
+      <c r="A15" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>Limpiar superficie de barra con desinfectante</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="F15" s="43" t="n"/>
+      <c r="G15" s="44" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="n">
+      <c r="A16" s="39" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Limpiar fregadero de barra (desatascar si necesario)</t>
-        </is>
-      </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Limpiar fregadero de barra (desatascar si hace falta)</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="15" t="n"/>
+      <c r="F16" s="43" t="n"/>
+      <c r="G16" s="44" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="32" t="n">
+      <c r="A17" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>Limpiar grifo de cerveza (purgar, limpiar boquilla)</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="15" t="n"/>
+      <c r="F17" s="43" t="n"/>
+      <c r="G17" s="44" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="n">
+      <c r="A18" s="39" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>Limpiar máquina de espresso (backflush, limpiar grupo)</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="15" t="n"/>
+      <c r="F18" s="43" t="n"/>
+      <c r="G18" s="44" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="n">
+      <c r="A19" s="39" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>Limpiar molinillo de café</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="15" t="n"/>
+      <c r="F19" s="43" t="n"/>
+      <c r="G19" s="44" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="n">
+      <c r="A20" s="39" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>Vaciar y limpiar lavavajillas de barra</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="15" t="n"/>
+      <c r="F20" s="43" t="n"/>
+      <c r="G20" s="44" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="n">
+      <c r="A21" s="39" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>Barrer y fregar suelo de barra (detrás de barra)</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="15" t="n"/>
-    </row>
-    <row r="22"/>
+      <c r="F21" s="43" t="n"/>
+      <c r="G21" s="44" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="45" t="n"/>
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="45" t="n"/>
+      <c r="E22" s="45" t="n"/>
+      <c r="F22" s="45" t="n"/>
+      <c r="G22" s="45" t="n"/>
+    </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="52" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cierre Administrativo</t>
         </is>
       </c>
-      <c r="B23" s="30" t="n"/>
-      <c r="C23" s="30" t="n"/>
-      <c r="D23" s="30" t="n"/>
-      <c r="E23" s="30" t="n"/>
-      <c r="F23" s="30" t="n"/>
-      <c r="G23" s="31" t="n"/>
+      <c r="B23" s="37" t="n"/>
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="37" t="n"/>
+      <c r="E23" s="37" t="n"/>
+      <c r="F23" s="37" t="n"/>
+      <c r="G23" s="38" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="32" t="n">
+      <c r="A24" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>Cuadrar caja / cierre de TPV</t>
-        </is>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>Comprobar que el arqueo del día ha quedado cerrado y firmado: el recuento no se repite aquí, se hace en «Cierre de Caja» del fichero 09-apertura-cierre-caja.xlsx</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="15" t="n"/>
+      <c r="F24" s="43" t="n"/>
+      <c r="G24" s="44" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="n">
+      <c r="A25" s="39" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="40" t="inlineStr">
         <is>
           <t>Registrar botellas abiertas (inventario rápido)</t>
         </is>
       </c>
-      <c r="C25" s="29" t="inlineStr">
+      <c r="C25" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="42" t="inlineStr">
         <is>
           <t>02:15</t>
         </is>
       </c>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="15" t="n"/>
+      <c r="F25" s="43" t="n"/>
+      <c r="G25" s="44" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="n">
+      <c r="A26" s="39" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>Anotar las mermas del turno (cristalería rota, derrames, cócteles devueltos y botella caída): sin este dato el pour cost del mes sale mal</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
+        <is>
+          <t>Bartender</t>
+        </is>
+      </c>
+      <c r="E26" s="42" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="F26" s="43" t="n"/>
+      <c r="G26" s="44" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>Anotar incidencias del turno (rotura, queja, falta stock)</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D27" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E27" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="15" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="32" t="n">
-        <v>18</v>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="F27" s="43" t="n"/>
+      <c r="G27" s="44" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>Apagar música, iluminación decorativa</t>
         </is>
       </c>
-      <c r="C27" s="29" t="inlineStr">
+      <c r="C28" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D28" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E28" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="15" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="32" t="n">
-        <v>19</v>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="F28" s="43" t="n"/>
+      <c r="G28" s="44" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="39" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>Verificar que no queda nadie en el local</t>
         </is>
       </c>
-      <c r="C28" s="29" t="inlineStr">
+      <c r="C29" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D29" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E29" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="15" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="32" t="n">
-        <v>20</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="F29" s="43" t="n"/>
+      <c r="G29" s="44" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>Activar alarma y cerrar con llave</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C30" s="41" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D30" s="42" t="inlineStr">
         <is>
           <t>Bartender</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E30" s="42" t="inlineStr">
         <is>
           <t>02:30</t>
         </is>
       </c>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="15" t="n"/>
-    </row>
-    <row r="30"/>
+      <c r="F30" s="43" t="n"/>
+      <c r="G30" s="44" t="n"/>
+    </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="45" t="n"/>
+      <c r="B31" s="45" t="n"/>
+      <c r="C31" s="45" t="n"/>
+      <c r="D31" s="45" t="n"/>
+      <c r="E31" s="45" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="45" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cierre Terraza</t>
         </is>
       </c>
-      <c r="B31" s="30" t="n"/>
-      <c r="C31" s="30" t="n"/>
-      <c r="D31" s="30" t="n"/>
-      <c r="E31" s="30" t="n"/>
-      <c r="F31" s="30" t="n"/>
-      <c r="G31" s="31" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="32" t="n">
-        <v>21</v>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="37" t="n"/>
+      <c r="G32" s="38" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="39" t="n">
+        <v>22</v>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
         <is>
           <t>Recoger mesas y sillas de terraza (o asegurar)</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C33" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D33" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E33" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F32" s="14" t="n"/>
-      <c r="G32" s="15" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="32" t="n">
-        <v>22</v>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="F33" s="43" t="n"/>
+      <c r="G33" s="44" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="39" t="n">
+        <v>23</v>
+      </c>
+      <c r="B34" s="40" t="inlineStr">
         <is>
           <t>Recoger ceniceros, cartas y servilleteros</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C34" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D34" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E34" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="15" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="32" t="n">
-        <v>23</v>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="F34" s="43" t="n"/>
+      <c r="G34" s="44" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="39" t="n">
+        <v>24</v>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
         <is>
           <t>Guardar sombrillas y cojines</t>
         </is>
       </c>
-      <c r="C34" s="20" t="inlineStr">
+      <c r="C35" s="41" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D35" s="42" t="inlineStr">
         <is>
           <t>Barback</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E35" s="42" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15" t="n"/>
-    </row>
-    <row r="35"/>
-    <row r="36"/>
+      <c r="F35" s="43" t="n"/>
+      <c r="G35" s="44" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="48" t="n"/>
+      <c r="B36" s="49" t="n"/>
+      <c r="C36" s="41" t="n"/>
+      <c r="D36" s="42" t="n"/>
+      <c r="E36" s="42" t="n"/>
+      <c r="F36" s="43" t="n"/>
+      <c r="G36" s="44" t="n"/>
+    </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="48" t="n"/>
+      <c r="B37" s="49" t="n"/>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="42" t="n"/>
+      <c r="E37" s="42" t="n"/>
+      <c r="F37" s="43" t="n"/>
+      <c r="G37" s="44" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="n"/>
+      <c r="B38" s="49" t="n"/>
+      <c r="C38" s="41" t="n"/>
+      <c r="D38" s="42" t="n"/>
+      <c r="E38" s="42" t="n"/>
+      <c r="F38" s="43" t="n"/>
+      <c r="G38" s="44" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="48" t="n"/>
+      <c r="B39" s="49" t="n"/>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="42" t="n"/>
+      <c r="E39" s="42" t="n"/>
+      <c r="F39" s="43" t="n"/>
+      <c r="G39" s="44" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="48" t="n"/>
+      <c r="B40" s="49" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="42" t="n"/>
+      <c r="E40" s="42" t="n"/>
+      <c r="F40" s="43" t="n"/>
+      <c r="G40" s="44" t="n"/>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="D37" s="21">
-        <f>COUNTIF(F5:F35,"✓")</f>
+      <c r="D42" s="21">
+        <f>COUNTIFS(B5:B40,"?*",F5:F40,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E37" s="22" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F37" s="21">
-        <f>COUNTIF(B5:B35,"?*")</f>
-        <v>23.0</v>
-      </c>
-    </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="F42" s="21">
+        <f>COUNTIF(B5:B40,"?*")-COUNTIF(F5:F40,"N/A")</f>
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>Verificado por:</t>
         </is>
       </c>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="30" t="n"/>
-      <c r="D39" s="31" t="n"/>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="B44" s="50" t="n"/>
+      <c r="C44" s="30" t="n"/>
+      <c r="D44" s="31" t="n"/>
+      <c r="E44" s="21" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="F39" s="15" t="n"/>
-      <c r="G39" s="31" t="n"/>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="23" t="inlineStr">
+      <c r="F44" s="50" t="n"/>
+      <c r="G44" s="31" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
         <is>
           <t>— Kit de Tareas Recurrentes · Bar / Cocktails · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="9">
+    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A23:G23"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F44:G44"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B44:D44"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G35">
+  <conditionalFormatting sqref="A5:G40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F32 F33 F34 F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F33 F34 F35 F36 F37 F38 F39 F40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>